<commit_message>
CSV finalizado com interface streamlit e criacao de tabelas oficiais do Excel
</commit_message>
<xml_diff>
--- a/relatorio.xlsx
+++ b/relatorio.xlsx
@@ -17,9 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="€#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="DD-MM-YYYY"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -69,16 +71,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -153,6 +157,31 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela_Dados_limpos" displayName="Tabela_Dados_limpos" ref="A1:E4" headerRowCount="1">
+  <autoFilter ref="A1:E4"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="data"/>
+    <tableColumn id="2" name="produto"/>
+    <tableColumn id="3" name="quantidade"/>
+    <tableColumn id="4" name="preco"/>
+    <tableColumn id="5" name="total_linha"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabela_Relatorio" displayName="Tabela_Relatorio" ref="A1:B19" headerRowCount="1">
+  <autoFilter ref="A1:B19"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Metrica"/>
+    <tableColumn id="2" name="Valor"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -485,18 +514,18 @@
       <c r="A2" s="2" t="n">
         <v>45658</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>camisola</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="5" t="n">
         <v>19.9</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="6" t="n">
         <v>39.8</v>
       </c>
     </row>
@@ -504,18 +533,18 @@
       <c r="A3" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>calções</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>24.5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="6" t="n">
         <v>24.5</v>
       </c>
     </row>
@@ -523,23 +552,26 @@
       <c r="A4" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>meias</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="5" t="n">
         <v>3.5</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="6" t="n">
         <v>17.5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -552,203 +584,233 @@
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="n"/>
-      <c r="B1" s="1" t="n">
-        <v>0</v>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metrica</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>linhas</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>3</v>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>colunas</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>4</v>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>total_quantidade</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>8</v>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>soma_precos_unitarios</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>47.9</v>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>47.9</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>total_faturado</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>81.8</v>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>81.8</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>media_preco</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>15.96666666666667</v>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>15.966666666666667</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>media_quantidade</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>2.666666666666667</v>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>2.6666666666666665</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>produto_mais_vendido</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>meias</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>quantidade_maxima</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>5</v>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>produto_mais_caro</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>calções</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>preco_maximo</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>24.5</v>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>primeira_data</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>45658</v>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2025-01-01 00:00:00</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ultima_data</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
-        <v>45660</v>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2025-01-03 00:00:00</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>produtos_unicos</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>3</v>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>produtos_vendidos_uma_vez</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>['calções']</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>top_3_produtos</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>1º meias - 5 unidades | 2º camisola - 2 unidades | 3º calções - 1 unidades</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>percentagens</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>meias: 62.50% | camisola: 25.00% | calções: 12.50%</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>nomes_colunas</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>data | produto | quantidade | preco | total_linha</t>
         </is>
@@ -756,5 +818,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>